<commit_message>
Update oil reserves by country.xlsx
</commit_message>
<xml_diff>
--- a/data/oil reserves by country.xlsx
+++ b/data/oil reserves by country.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PB\oil-reserves-by-country\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEDC4C11-2D0F-4987-BFD7-1C60C005286D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F7426A2-B88B-4D0A-8A1C-4DF133FB1490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{57AD8D99-2A58-4150-8F43-2E7CA4794407}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="75">
   <si>
     <t>OECD Americas</t>
   </si>
@@ -234,9 +234,6 @@
     <t>2024</t>
   </si>
   <si>
-    <t>Total</t>
-  </si>
-  <si>
     <t>Country</t>
   </si>
   <si>
@@ -262,13 +259,20 @@
   </si>
   <si>
     <t>Rank</t>
+  </si>
+  <si>
+    <t>Total World</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -278,6 +282,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -302,17 +313,157 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="12">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -329,19 +480,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{81CF8948-434B-4C23-B0AE-7ADD51952A08}" name="Table1" displayName="Table1" ref="B1:L45" totalsRowCount="1">
   <autoFilter ref="B1:L44" xr:uid="{81CF8948-434B-4C23-B0AE-7ADD51952A08}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:L44">
-    <sortCondition descending="1" ref="I1:I44"/>
+    <sortCondition ref="C1:C44"/>
   </sortState>
   <tableColumns count="11">
     <tableColumn id="10" xr3:uid="{673E017D-9321-42FB-9E51-E001EB12060E}" name="Sl_Org"/>
     <tableColumn id="11" xr3:uid="{DA8B90E1-62B1-4DBE-AA03-E7920051888C}" name="Rank"/>
-    <tableColumn id="1" xr3:uid="{0CEDEDC5-7C6A-4011-930E-40AD3B2B1861}" name="Country" totalsRowLabel="Total"/>
-    <tableColumn id="2" xr3:uid="{591E2852-2407-4C86-8C64-EB297AB9ED70}" name="2020" totalsRowFunction="sum"/>
-    <tableColumn id="3" xr3:uid="{D9003A69-DAD0-460C-9922-0296A3B8DF39}" name="2021" totalsRowFunction="sum"/>
-    <tableColumn id="4" xr3:uid="{671B216A-5BE7-40BA-B9F0-8F976B44EB61}" name="2022" totalsRowFunction="sum"/>
-    <tableColumn id="5" xr3:uid="{7E050318-17B1-45AB-9BE9-1A52C3BE4D0B}" name="2023" totalsRowFunction="sum"/>
-    <tableColumn id="6" xr3:uid="{884D50D5-E95B-4627-A909-4866F345DD84}" name="2024" totalsRowFunction="sum"/>
-    <tableColumn id="7" xr3:uid="{080DB9F4-1626-4937-89FD-46B4596B0C1A}" name="change24/23" totalsRowFunction="sum"/>
-    <tableColumn id="8" xr3:uid="{8136C249-7D1D-47DE-9F22-B69EA9E74A70}" name="Country2" totalsRowFunction="sum"/>
+    <tableColumn id="1" xr3:uid="{0CEDEDC5-7C6A-4011-930E-40AD3B2B1861}" name="Country" totalsRowLabel="Total World"/>
+    <tableColumn id="2" xr3:uid="{591E2852-2407-4C86-8C64-EB297AB9ED70}" name="2020" totalsRowFunction="sum" dataDxfId="11" totalsRowDxfId="8" dataCellStyle="Comma" totalsRowCellStyle="Comma"/>
+    <tableColumn id="3" xr3:uid="{D9003A69-DAD0-460C-9922-0296A3B8DF39}" name="2021" totalsRowFunction="sum" dataDxfId="10" totalsRowDxfId="7" dataCellStyle="Comma" totalsRowCellStyle="Comma"/>
+    <tableColumn id="4" xr3:uid="{671B216A-5BE7-40BA-B9F0-8F976B44EB61}" name="2022" totalsRowFunction="sum" dataDxfId="9" totalsRowDxfId="6" dataCellStyle="Comma" totalsRowCellStyle="Comma"/>
+    <tableColumn id="5" xr3:uid="{7E050318-17B1-45AB-9BE9-1A52C3BE4D0B}" name="2023" totalsRowFunction="sum" dataDxfId="3" totalsRowDxfId="5" dataCellStyle="Comma" totalsRowCellStyle="Comma"/>
+    <tableColumn id="6" xr3:uid="{884D50D5-E95B-4627-A909-4866F345DD84}" name="2024" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0" dataCellStyle="Comma" totalsRowCellStyle="Comma"/>
+    <tableColumn id="7" xr3:uid="{080DB9F4-1626-4937-89FD-46B4596B0C1A}" name="change24/23" totalsRowFunction="sum" dataDxfId="2" totalsRowDxfId="4" dataCellStyle="Comma" totalsRowCellStyle="Comma"/>
+    <tableColumn id="8" xr3:uid="{8136C249-7D1D-47DE-9F22-B69EA9E74A70}" name="Country2"/>
     <tableColumn id="9" xr3:uid="{DB111182-2EE3-4492-B4C0-1A616573A28F}" name="Continent"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2324,47 +2475,51 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8D51AE7-6A31-478B-92C5-3FDADD0E5BE5}">
-  <dimension ref="B1:L47"/>
+  <dimension ref="B1:L46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.7109375" customWidth="1"/>
-    <col min="4" max="10" width="15.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="8" width="15.5703125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" style="3" customWidth="1"/>
+    <col min="10" max="10" width="15.5703125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C1" t="s">
         <v>73</v>
       </c>
-      <c r="C1" t="s">
-        <v>74</v>
-      </c>
       <c r="D1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="K1" t="s">
+        <v>71</v>
+      </c>
+      <c r="L1" t="s">
         <v>66</v>
-      </c>
-      <c r="E1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G1" t="s">
-        <v>62</v>
-      </c>
-      <c r="H1" t="s">
-        <v>63</v>
-      </c>
-      <c r="I1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" t="s">
-        <v>59</v>
-      </c>
-      <c r="K1" t="s">
-        <v>72</v>
-      </c>
-      <c r="L1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
@@ -2377,29 +2532,29 @@
       <c r="D2" t="s">
         <v>24</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="2">
         <v>303561</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="2">
         <v>303468</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="2">
         <v>303221</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="2">
         <v>303008</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="3">
         <v>303221</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="2">
         <v>213</v>
       </c>
       <c r="K2">
         <v>1</v>
       </c>
       <c r="L2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
@@ -2412,29 +2567,29 @@
       <c r="D3" t="s">
         <v>31</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="2">
         <v>267082</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="2">
         <v>267192</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="2">
         <v>267192</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="2">
         <v>267230</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="3">
         <v>267200</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="2">
         <v>-30</v>
       </c>
       <c r="K3">
         <v>1</v>
       </c>
       <c r="L3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
@@ -2447,29 +2602,29 @@
       <c r="D4" t="s">
         <v>26</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="2">
         <v>208600</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="2">
         <v>208600</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="2">
         <v>208600</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="2">
         <v>208600</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="3">
         <v>208600</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="2">
         <v>0</v>
       </c>
       <c r="K4">
         <v>1</v>
       </c>
       <c r="L4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
@@ -2482,29 +2637,29 @@
       <c r="D5" t="s">
         <v>27</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="2">
         <v>145019</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="2">
         <v>145019</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="2">
         <v>145019</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="2">
         <v>145019</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="3">
         <v>145019</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="2">
         <v>0</v>
       </c>
       <c r="K5">
         <v>1</v>
       </c>
       <c r="L5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
@@ -2517,29 +2672,29 @@
       <c r="D6" t="s">
         <v>32</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="2">
         <v>107000</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="2">
         <v>111000</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="2">
         <v>113000</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="2">
         <v>113000</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="3">
         <v>113000</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="2">
         <v>0</v>
       </c>
       <c r="K6">
         <v>1</v>
       </c>
       <c r="L6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
@@ -2552,29 +2707,29 @@
       <c r="D7" t="s">
         <v>28</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="2">
         <v>101500</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="2">
         <v>101500</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="2">
         <v>101500</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="2">
         <v>101500</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="3">
         <v>101500</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="2">
         <v>0</v>
       </c>
       <c r="K7">
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
@@ -2587,29 +2742,29 @@
       <c r="D8" t="s">
         <v>43</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="2">
         <v>80000</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="2">
         <v>80000</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="2">
         <v>80000</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="2">
         <v>80000</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="3">
         <v>80000</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="2">
         <v>0</v>
       </c>
       <c r="K8">
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
@@ -2622,22 +2777,22 @@
       <c r="D9" t="s">
         <v>40</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="2">
         <v>48363</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="2">
         <v>48363</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="2">
         <v>48363</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="2">
         <v>48363</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="3">
         <v>48363</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="2">
         <v>0</v>
       </c>
       <c r="K9">
@@ -2657,29 +2812,29 @@
       <c r="D10" t="s">
         <v>4</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="2">
         <v>35835</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="2">
         <v>41610</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="2">
         <v>45271</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="2">
         <v>43492</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="3">
         <v>45014</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="2">
         <v>1522</v>
       </c>
       <c r="K10">
         <v>1</v>
       </c>
       <c r="L10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
@@ -2692,22 +2847,22 @@
       <c r="D11" t="s">
         <v>41</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="2">
         <v>36910</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="2">
         <v>37050</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="2">
         <v>36967</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="2">
         <v>37500</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="3">
         <v>37280</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="2">
         <v>-220</v>
       </c>
       <c r="K11">
@@ -2727,29 +2882,29 @@
       <c r="D12" t="s">
         <v>47</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="2">
         <v>30000</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="2">
         <v>30000</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="2">
         <v>30000</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="2">
         <v>30000</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="3">
         <v>30000</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="2">
         <v>0</v>
       </c>
       <c r="K12">
         <v>1</v>
       </c>
       <c r="L12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
@@ -2762,719 +2917,722 @@
       <c r="D13" t="s">
         <v>12</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="2">
         <v>26023</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="2">
         <v>26491</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="2">
         <v>27003</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="2">
         <v>27889</v>
       </c>
-      <c r="I13">
+      <c r="I13" s="3">
         <v>28182</v>
       </c>
-      <c r="J13">
+      <c r="J13" s="2">
         <v>293</v>
       </c>
       <c r="K13">
         <v>1</v>
       </c>
       <c r="L13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="C14">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14">
-        <v>17027</v>
-      </c>
-      <c r="F14">
-        <v>28037</v>
-      </c>
-      <c r="G14">
-        <v>27585</v>
-      </c>
-      <c r="H14">
-        <v>27507</v>
-      </c>
-      <c r="I14">
-        <v>27541</v>
-      </c>
-      <c r="J14">
-        <v>34</v>
+        <v>30</v>
+      </c>
+      <c r="E14" s="2">
+        <v>25244</v>
+      </c>
+      <c r="F14" s="2">
+        <v>25244</v>
+      </c>
+      <c r="G14" s="2">
+        <v>25244</v>
+      </c>
+      <c r="H14" s="2">
+        <v>25244</v>
+      </c>
+      <c r="I14" s="3">
+        <v>25244</v>
+      </c>
+      <c r="J14" s="2">
+        <v>0</v>
       </c>
       <c r="K14">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="L14" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="C15">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D15" t="s">
-        <v>30</v>
-      </c>
-      <c r="E15">
-        <v>25244</v>
-      </c>
-      <c r="F15">
-        <v>25244</v>
-      </c>
-      <c r="G15">
-        <v>25244</v>
-      </c>
-      <c r="H15">
-        <v>25244</v>
-      </c>
-      <c r="I15">
-        <v>25244</v>
-      </c>
-      <c r="J15">
-        <v>0</v>
+        <v>21</v>
+      </c>
+      <c r="E15" s="2">
+        <v>12715</v>
+      </c>
+      <c r="F15" s="2">
+        <v>11890</v>
+      </c>
+      <c r="G15" s="2">
+        <v>13242</v>
+      </c>
+      <c r="H15" s="2">
+        <v>14856</v>
+      </c>
+      <c r="I15" s="3">
+        <v>15894</v>
+      </c>
+      <c r="J15" s="2">
+        <v>1038</v>
       </c>
       <c r="K15">
         <v>1</v>
       </c>
       <c r="L15" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="C16">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D16" t="s">
-        <v>21</v>
-      </c>
-      <c r="E16">
-        <v>12715</v>
-      </c>
-      <c r="F16">
-        <v>11890</v>
-      </c>
-      <c r="G16">
-        <v>13242</v>
-      </c>
-      <c r="H16">
-        <v>14856</v>
-      </c>
-      <c r="I16">
-        <v>15894</v>
-      </c>
-      <c r="J16">
-        <v>1038</v>
+        <v>34</v>
+      </c>
+      <c r="E16" s="2">
+        <v>12200</v>
+      </c>
+      <c r="F16" s="2">
+        <v>12200</v>
+      </c>
+      <c r="G16" s="2">
+        <v>12200</v>
+      </c>
+      <c r="H16" s="2">
+        <v>12200</v>
+      </c>
+      <c r="I16" s="3">
+        <v>12200</v>
+      </c>
+      <c r="J16" s="2">
+        <v>0</v>
       </c>
       <c r="K16">
         <v>1</v>
       </c>
       <c r="L16" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="C17">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D17" t="s">
-        <v>34</v>
-      </c>
-      <c r="E17">
-        <v>12200</v>
-      </c>
-      <c r="F17">
-        <v>12200</v>
-      </c>
-      <c r="G17">
-        <v>12200</v>
-      </c>
-      <c r="H17">
-        <v>12200</v>
-      </c>
-      <c r="I17">
-        <v>12200</v>
-      </c>
-      <c r="J17">
+        <v>23</v>
+      </c>
+      <c r="E17" s="2">
+        <v>8273</v>
+      </c>
+      <c r="F17" s="2">
+        <v>8273</v>
+      </c>
+      <c r="G17" s="2">
+        <v>8273</v>
+      </c>
+      <c r="H17" s="2">
+        <v>8273</v>
+      </c>
+      <c r="I17" s="3">
+        <v>8273</v>
+      </c>
+      <c r="J17" s="2">
         <v>0</v>
       </c>
       <c r="K17">
         <v>1</v>
       </c>
       <c r="L17" t="s">
-        <v>33</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18">
-        <v>34</v>
+        <v>66</v>
       </c>
       <c r="C18">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D18" t="s">
-        <v>23</v>
-      </c>
-      <c r="E18">
-        <v>8273</v>
-      </c>
-      <c r="F18">
-        <v>8273</v>
-      </c>
-      <c r="G18">
-        <v>8273</v>
-      </c>
-      <c r="H18">
-        <v>8273</v>
-      </c>
-      <c r="I18">
-        <v>8273</v>
-      </c>
-      <c r="J18">
+        <v>45</v>
+      </c>
+      <c r="E18" s="2">
+        <v>7000</v>
+      </c>
+      <c r="F18" s="2">
+        <v>7000</v>
+      </c>
+      <c r="G18" s="2">
+        <v>7000</v>
+      </c>
+      <c r="H18" s="2">
+        <v>7000</v>
+      </c>
+      <c r="I18" s="3">
+        <v>7000</v>
+      </c>
+      <c r="J18" s="2">
         <v>0</v>
       </c>
       <c r="K18">
         <v>1</v>
       </c>
       <c r="L18" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19">
-        <v>66</v>
+        <v>11</v>
       </c>
       <c r="C19">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D19" t="s">
-        <v>45</v>
-      </c>
-      <c r="E19">
-        <v>7000</v>
-      </c>
-      <c r="F19">
-        <v>7000</v>
-      </c>
-      <c r="G19">
-        <v>7000</v>
-      </c>
-      <c r="H19">
-        <v>7000</v>
-      </c>
-      <c r="I19">
-        <v>7000</v>
-      </c>
-      <c r="J19">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="E19" s="2">
+        <v>7902</v>
+      </c>
+      <c r="F19" s="2">
+        <v>7745</v>
+      </c>
+      <c r="G19" s="2">
+        <v>7573</v>
+      </c>
+      <c r="H19" s="2">
+        <v>7642</v>
+      </c>
+      <c r="I19" s="3">
+        <v>6912</v>
+      </c>
+      <c r="J19" s="2">
+        <v>-730</v>
       </c>
       <c r="K19">
         <v>1</v>
       </c>
       <c r="L19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C20">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D20" t="s">
-        <v>7</v>
-      </c>
-      <c r="E20">
-        <v>7902</v>
-      </c>
-      <c r="F20">
-        <v>7745</v>
-      </c>
-      <c r="G20">
-        <v>7573</v>
-      </c>
-      <c r="H20">
-        <v>7642</v>
-      </c>
-      <c r="I20">
-        <v>6912</v>
-      </c>
-      <c r="J20">
-        <v>-730</v>
+        <v>3</v>
+      </c>
+      <c r="E20" s="2">
+        <v>5498</v>
+      </c>
+      <c r="F20" s="2">
+        <v>5618</v>
+      </c>
+      <c r="G20" s="2">
+        <v>5558</v>
+      </c>
+      <c r="H20" s="2">
+        <v>5293</v>
+      </c>
+      <c r="I20" s="3">
+        <v>5136</v>
+      </c>
+      <c r="J20" s="2">
+        <v>-157</v>
       </c>
       <c r="K20">
         <v>1</v>
       </c>
       <c r="L20" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21">
-        <v>5</v>
+        <v>59</v>
       </c>
       <c r="C21">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D21" t="s">
-        <v>3</v>
-      </c>
-      <c r="E21">
-        <v>5498</v>
-      </c>
-      <c r="F21">
-        <v>5618</v>
-      </c>
-      <c r="G21">
-        <v>5558</v>
-      </c>
-      <c r="H21">
-        <v>5293</v>
-      </c>
-      <c r="I21">
-        <v>5136</v>
-      </c>
-      <c r="J21">
-        <v>-157</v>
+        <v>42</v>
+      </c>
+      <c r="E21" s="2">
+        <v>5000</v>
+      </c>
+      <c r="F21" s="2">
+        <v>5000</v>
+      </c>
+      <c r="G21" s="2">
+        <v>5000</v>
+      </c>
+      <c r="H21" s="2">
+        <v>5000</v>
+      </c>
+      <c r="I21" s="3">
+        <v>5000</v>
+      </c>
+      <c r="J21" s="2">
+        <v>0</v>
       </c>
       <c r="K21">
         <v>1</v>
       </c>
       <c r="L21" t="s">
-        <v>68</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="C22">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D22" t="s">
-        <v>42</v>
-      </c>
-      <c r="E22">
-        <v>5000</v>
-      </c>
-      <c r="F22">
-        <v>5000</v>
-      </c>
-      <c r="G22">
-        <v>5000</v>
-      </c>
-      <c r="H22">
-        <v>5000</v>
-      </c>
-      <c r="I22">
-        <v>5000</v>
-      </c>
-      <c r="J22">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="E22" s="2">
+        <v>4605</v>
+      </c>
+      <c r="F22" s="2">
+        <v>4489</v>
+      </c>
+      <c r="G22" s="2">
+        <v>4370</v>
+      </c>
+      <c r="H22" s="2">
+        <v>4849</v>
+      </c>
+      <c r="I22" s="3">
+        <v>4981</v>
+      </c>
+      <c r="J22" s="2">
+        <v>132</v>
       </c>
       <c r="K22">
         <v>1</v>
       </c>
       <c r="L22" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="C23">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D23" t="s">
-        <v>13</v>
-      </c>
-      <c r="E23">
-        <v>4605</v>
-      </c>
-      <c r="F23">
-        <v>4489</v>
-      </c>
-      <c r="G23">
-        <v>4370</v>
-      </c>
-      <c r="H23">
-        <v>4849</v>
-      </c>
-      <c r="I23">
-        <v>4981</v>
-      </c>
-      <c r="J23">
-        <v>132</v>
+        <v>29</v>
+      </c>
+      <c r="E23" s="2">
+        <v>5373</v>
+      </c>
+      <c r="F23" s="2">
+        <v>5373</v>
+      </c>
+      <c r="G23" s="2">
+        <v>4856</v>
+      </c>
+      <c r="H23" s="2">
+        <v>4905</v>
+      </c>
+      <c r="I23" s="3">
+        <v>4971</v>
+      </c>
+      <c r="J23" s="2">
+        <v>66</v>
       </c>
       <c r="K23">
         <v>1</v>
       </c>
       <c r="L23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="C24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D24" t="s">
-        <v>29</v>
-      </c>
-      <c r="E24">
-        <v>5373</v>
-      </c>
-      <c r="F24">
-        <v>5373</v>
-      </c>
-      <c r="G24">
-        <v>4856</v>
-      </c>
-      <c r="H24">
-        <v>4905</v>
-      </c>
-      <c r="I24">
-        <v>4971</v>
-      </c>
-      <c r="J24">
-        <v>66</v>
+        <v>18</v>
+      </c>
+      <c r="E24" s="2">
+        <v>4400</v>
+      </c>
+      <c r="F24" s="2">
+        <v>4400</v>
+      </c>
+      <c r="G24" s="2">
+        <v>4400</v>
+      </c>
+      <c r="H24" s="2">
+        <v>4400</v>
+      </c>
+      <c r="I24" s="3">
+        <v>4400</v>
+      </c>
+      <c r="J24" s="2">
+        <v>0</v>
       </c>
       <c r="K24">
         <v>1</v>
       </c>
       <c r="L24" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="C25">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D25" t="s">
-        <v>18</v>
-      </c>
-      <c r="E25">
-        <v>4400</v>
-      </c>
-      <c r="F25">
-        <v>4400</v>
-      </c>
-      <c r="G25">
-        <v>4400</v>
-      </c>
-      <c r="H25">
-        <v>4400</v>
-      </c>
-      <c r="I25">
-        <v>4400</v>
-      </c>
-      <c r="J25">
+        <v>1</v>
+      </c>
+      <c r="E25" s="2">
+        <v>4299</v>
+      </c>
+      <c r="F25" s="2">
+        <v>4817</v>
+      </c>
+      <c r="G25" s="2">
+        <v>4363</v>
+      </c>
+      <c r="H25" s="2">
+        <v>4344</v>
+      </c>
+      <c r="I25" s="3">
+        <v>4344</v>
+      </c>
+      <c r="J25" s="2">
         <v>0</v>
       </c>
       <c r="K25">
         <v>1</v>
       </c>
       <c r="L25" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26">
-        <v>3</v>
+        <v>54</v>
       </c>
       <c r="C26">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D26" t="s">
-        <v>1</v>
-      </c>
-      <c r="E26">
-        <v>4299</v>
-      </c>
-      <c r="F26">
-        <v>4817</v>
-      </c>
-      <c r="G26">
-        <v>4363</v>
-      </c>
-      <c r="H26">
-        <v>4344</v>
-      </c>
-      <c r="I26">
-        <v>4344</v>
-      </c>
-      <c r="J26">
+        <v>37</v>
+      </c>
+      <c r="E26" s="2">
+        <v>3075</v>
+      </c>
+      <c r="F26" s="2">
+        <v>3300</v>
+      </c>
+      <c r="G26" s="2">
+        <v>3300</v>
+      </c>
+      <c r="H26" s="2">
+        <v>3300</v>
+      </c>
+      <c r="I26" s="3">
+        <v>3300</v>
+      </c>
+      <c r="J26" s="2">
         <v>0</v>
       </c>
       <c r="K26">
         <v>1</v>
       </c>
       <c r="L26" t="s">
-        <v>68</v>
+        <v>33</v>
       </c>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="C27">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D27" t="s">
-        <v>37</v>
-      </c>
-      <c r="E27">
-        <v>3075</v>
-      </c>
-      <c r="F27">
-        <v>3300</v>
-      </c>
-      <c r="G27">
-        <v>3300</v>
-      </c>
-      <c r="H27">
-        <v>3300</v>
-      </c>
-      <c r="I27">
-        <v>3300</v>
-      </c>
-      <c r="J27">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="E27" s="2">
+        <v>2483</v>
+      </c>
+      <c r="F27" s="2">
+        <v>2411</v>
+      </c>
+      <c r="G27" s="2">
+        <v>2838</v>
+      </c>
+      <c r="H27" s="2">
+        <v>2924</v>
+      </c>
+      <c r="I27" s="3">
+        <v>2999</v>
+      </c>
+      <c r="J27" s="2">
+        <v>75</v>
       </c>
       <c r="K27">
         <v>1</v>
       </c>
       <c r="L27" t="s">
-        <v>33</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C28">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D28" t="s">
-        <v>20</v>
-      </c>
-      <c r="E28">
-        <v>2483</v>
-      </c>
-      <c r="F28">
-        <v>2411</v>
-      </c>
-      <c r="G28">
-        <v>2838</v>
-      </c>
-      <c r="H28">
-        <v>2924</v>
-      </c>
-      <c r="I28">
-        <v>2999</v>
-      </c>
-      <c r="J28">
-        <v>75</v>
+        <v>17</v>
+      </c>
+      <c r="E28" s="2">
+        <v>3600</v>
+      </c>
+      <c r="F28" s="2">
+        <v>3600</v>
+      </c>
+      <c r="G28" s="2">
+        <v>2700</v>
+      </c>
+      <c r="H28" s="2">
+        <v>2700</v>
+      </c>
+      <c r="I28" s="3">
+        <v>2700</v>
+      </c>
+      <c r="J28" s="2">
+        <v>0</v>
       </c>
       <c r="K28">
         <v>1</v>
       </c>
       <c r="L28" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="C29">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D29" t="s">
-        <v>17</v>
-      </c>
-      <c r="E29">
-        <v>3600</v>
-      </c>
-      <c r="F29">
-        <v>3600</v>
-      </c>
-      <c r="G29">
-        <v>2700</v>
-      </c>
-      <c r="H29">
-        <v>2700</v>
-      </c>
-      <c r="I29">
-        <v>2700</v>
-      </c>
-      <c r="J29">
+        <v>35</v>
+      </c>
+      <c r="E29" s="2">
+        <v>7231</v>
+      </c>
+      <c r="F29" s="2">
+        <v>2516</v>
+      </c>
+      <c r="G29" s="2">
+        <v>2550</v>
+      </c>
+      <c r="H29" s="2">
+        <v>2550</v>
+      </c>
+      <c r="I29" s="3">
+        <v>2550</v>
+      </c>
+      <c r="J29" s="2">
         <v>0</v>
       </c>
       <c r="K29">
         <v>1</v>
       </c>
       <c r="L29" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="C30">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D30" t="s">
-        <v>35</v>
-      </c>
-      <c r="E30">
-        <v>7231</v>
-      </c>
-      <c r="F30">
-        <v>2516</v>
-      </c>
-      <c r="G30">
-        <v>2550</v>
-      </c>
-      <c r="H30">
-        <v>2550</v>
-      </c>
-      <c r="I30">
-        <v>2550</v>
-      </c>
-      <c r="J30">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="E30" s="2">
+        <v>2480</v>
+      </c>
+      <c r="F30" s="2">
+        <v>2440</v>
+      </c>
+      <c r="G30" s="2">
+        <v>2250</v>
+      </c>
+      <c r="H30" s="2">
+        <v>2270</v>
+      </c>
+      <c r="I30" s="3">
+        <v>2410</v>
+      </c>
+      <c r="J30" s="2">
+        <v>140</v>
       </c>
       <c r="K30">
         <v>1</v>
       </c>
       <c r="L30" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C31">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D31" t="s">
-        <v>16</v>
-      </c>
-      <c r="E31">
-        <v>2480</v>
-      </c>
-      <c r="F31">
-        <v>2440</v>
-      </c>
-      <c r="G31">
-        <v>2250</v>
-      </c>
-      <c r="H31">
-        <v>2270</v>
-      </c>
-      <c r="I31">
-        <v>2410</v>
-      </c>
-      <c r="J31">
-        <v>140</v>
+        <v>22</v>
+      </c>
+      <c r="E31" s="2">
+        <v>2036</v>
+      </c>
+      <c r="F31" s="2">
+        <v>1820</v>
+      </c>
+      <c r="G31" s="2">
+        <v>2040</v>
+      </c>
+      <c r="H31" s="2">
+        <v>2074</v>
+      </c>
+      <c r="I31" s="3">
+        <v>2019</v>
+      </c>
+      <c r="J31" s="2">
+        <v>-55</v>
       </c>
       <c r="K31">
         <v>1</v>
       </c>
       <c r="L31" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32">
+        <v>56</v>
+      </c>
+      <c r="C32">
+        <v>31</v>
+      </c>
+      <c r="D32" t="s">
+        <v>39</v>
+      </c>
+      <c r="E32" s="2">
+        <v>2000</v>
+      </c>
+      <c r="F32" s="2">
+        <v>2000</v>
+      </c>
+      <c r="G32" s="2">
+        <v>2000</v>
+      </c>
+      <c r="H32" s="2">
+        <v>2000</v>
+      </c>
+      <c r="I32" s="3">
+        <v>2000</v>
+      </c>
+      <c r="J32" s="2">
+        <v>0</v>
+      </c>
+      <c r="K32">
+        <v>1</v>
+      </c>
+      <c r="L32" t="s">
         <v>33</v>
-      </c>
-      <c r="C32">
-        <v>30</v>
-      </c>
-      <c r="D32" t="s">
-        <v>22</v>
-      </c>
-      <c r="E32">
-        <v>2036</v>
-      </c>
-      <c r="F32">
-        <v>1820</v>
-      </c>
-      <c r="G32">
-        <v>2040</v>
-      </c>
-      <c r="H32">
-        <v>2074</v>
-      </c>
-      <c r="I32">
-        <v>2019</v>
-      </c>
-      <c r="J32">
-        <v>-55</v>
-      </c>
-      <c r="K32">
-        <v>1</v>
-      </c>
-      <c r="L32" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C33">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D33" t="s">
-        <v>39</v>
-      </c>
-      <c r="E33">
-        <v>2000</v>
-      </c>
-      <c r="F33">
-        <v>2000</v>
-      </c>
-      <c r="G33">
-        <v>2000</v>
-      </c>
-      <c r="H33">
-        <v>2000</v>
-      </c>
-      <c r="I33">
-        <v>2000</v>
-      </c>
-      <c r="J33">
+        <v>36</v>
+      </c>
+      <c r="E33" s="2">
+        <v>1811</v>
+      </c>
+      <c r="F33" s="2">
+        <v>1811</v>
+      </c>
+      <c r="G33" s="2">
+        <v>1811</v>
+      </c>
+      <c r="H33" s="2">
+        <v>1811</v>
+      </c>
+      <c r="I33" s="3">
+        <v>1811</v>
+      </c>
+      <c r="J33" s="2">
         <v>0</v>
       </c>
       <c r="K33">
@@ -3486,100 +3644,100 @@
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="C34">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D34" t="s">
-        <v>36</v>
-      </c>
-      <c r="E34">
-        <v>1811</v>
-      </c>
-      <c r="F34">
-        <v>1811</v>
-      </c>
-      <c r="G34">
-        <v>1811</v>
-      </c>
-      <c r="H34">
-        <v>1811</v>
-      </c>
-      <c r="I34">
-        <v>1811</v>
-      </c>
-      <c r="J34">
+        <v>11</v>
+      </c>
+      <c r="E34" s="2">
+        <v>2390</v>
+      </c>
+      <c r="F34" s="2">
+        <v>1747</v>
+      </c>
+      <c r="G34" s="2">
+        <v>1803</v>
+      </c>
+      <c r="H34" s="2">
+        <v>1803</v>
+      </c>
+      <c r="I34" s="3">
+        <v>1803</v>
+      </c>
+      <c r="J34" s="2">
         <v>0</v>
       </c>
       <c r="K34">
         <v>1</v>
       </c>
       <c r="L34" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C35">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E35">
-        <v>2390</v>
-      </c>
-      <c r="F35">
-        <v>1747</v>
-      </c>
-      <c r="G35">
-        <v>1803</v>
-      </c>
-      <c r="H35">
-        <v>1803</v>
-      </c>
-      <c r="I35">
-        <v>1803</v>
-      </c>
-      <c r="J35">
+        <v>8</v>
+      </c>
+      <c r="E35" s="2">
+        <v>2500</v>
+      </c>
+      <c r="F35" s="2">
+        <v>2000</v>
+      </c>
+      <c r="G35" s="2">
+        <v>1800</v>
+      </c>
+      <c r="H35" s="2">
+        <v>1500</v>
+      </c>
+      <c r="I35" s="3">
+        <v>1500</v>
+      </c>
+      <c r="J35" s="2">
         <v>0</v>
       </c>
       <c r="K35">
         <v>1</v>
       </c>
       <c r="L35" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C36">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D36" t="s">
-        <v>8</v>
-      </c>
-      <c r="E36">
-        <v>2500</v>
-      </c>
-      <c r="F36">
-        <v>2000</v>
-      </c>
-      <c r="G36">
-        <v>1800</v>
-      </c>
-      <c r="H36">
-        <v>1500</v>
-      </c>
-      <c r="I36">
-        <v>1500</v>
-      </c>
-      <c r="J36">
+        <v>15</v>
+      </c>
+      <c r="E36" s="2">
+        <v>1100</v>
+      </c>
+      <c r="F36" s="2">
+        <v>1100</v>
+      </c>
+      <c r="G36" s="2">
+        <v>1100</v>
+      </c>
+      <c r="H36" s="2">
+        <v>1100</v>
+      </c>
+      <c r="I36" s="3">
+        <v>1100</v>
+      </c>
+      <c r="J36" s="2">
         <v>0</v>
       </c>
       <c r="K36">
@@ -3591,206 +3749,206 @@
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="C37">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D37" t="s">
-        <v>15</v>
-      </c>
-      <c r="E37">
+        <v>38</v>
+      </c>
+      <c r="E37" s="2">
         <v>1100</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="2">
         <v>1100</v>
       </c>
-      <c r="G37">
+      <c r="G37" s="2">
         <v>1100</v>
       </c>
-      <c r="H37">
+      <c r="H37" s="2">
         <v>1100</v>
       </c>
-      <c r="I37">
+      <c r="I37" s="3">
         <v>1100</v>
       </c>
-      <c r="J37">
+      <c r="J37" s="2">
         <v>0</v>
       </c>
       <c r="K37">
         <v>1</v>
       </c>
       <c r="L37" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="C38">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D38" t="s">
-        <v>38</v>
-      </c>
-      <c r="E38">
-        <v>1100</v>
-      </c>
-      <c r="F38">
-        <v>1100</v>
-      </c>
-      <c r="G38">
-        <v>1100</v>
-      </c>
-      <c r="H38">
-        <v>1100</v>
-      </c>
-      <c r="I38">
-        <v>1100</v>
-      </c>
-      <c r="J38">
+        <v>48</v>
+      </c>
+      <c r="E38" s="2">
+        <v>600</v>
+      </c>
+      <c r="F38" s="2">
+        <v>600</v>
+      </c>
+      <c r="G38" s="2">
+        <v>600</v>
+      </c>
+      <c r="H38" s="2">
+        <v>600</v>
+      </c>
+      <c r="I38" s="3">
+        <v>600</v>
+      </c>
+      <c r="J38" s="2">
         <v>0</v>
       </c>
       <c r="K38">
         <v>1</v>
       </c>
       <c r="L38" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C39">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D39" t="s">
-        <v>48</v>
-      </c>
-      <c r="E39">
-        <v>600</v>
-      </c>
-      <c r="F39">
-        <v>600</v>
-      </c>
-      <c r="G39">
-        <v>600</v>
-      </c>
-      <c r="H39">
-        <v>600</v>
-      </c>
-      <c r="I39">
-        <v>600</v>
-      </c>
-      <c r="J39">
+        <v>50</v>
+      </c>
+      <c r="E39" s="2">
+        <v>594</v>
+      </c>
+      <c r="F39" s="2">
+        <v>594</v>
+      </c>
+      <c r="G39" s="2">
+        <v>594</v>
+      </c>
+      <c r="H39" s="2">
+        <v>594</v>
+      </c>
+      <c r="I39" s="3">
+        <v>594</v>
+      </c>
+      <c r="J39" s="2">
         <v>0</v>
       </c>
       <c r="K39">
         <v>1</v>
       </c>
       <c r="L39" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C40">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D40" t="s">
-        <v>50</v>
-      </c>
-      <c r="E40">
-        <v>594</v>
-      </c>
-      <c r="F40">
-        <v>594</v>
-      </c>
-      <c r="G40">
-        <v>594</v>
-      </c>
-      <c r="H40">
-        <v>594</v>
-      </c>
-      <c r="I40">
-        <v>594</v>
-      </c>
-      <c r="J40">
+        <v>49</v>
+      </c>
+      <c r="E40" s="2">
+        <v>395</v>
+      </c>
+      <c r="F40" s="2">
+        <v>395</v>
+      </c>
+      <c r="G40" s="2">
+        <v>395</v>
+      </c>
+      <c r="H40" s="2">
+        <v>395</v>
+      </c>
+      <c r="I40" s="3">
+        <v>395</v>
+      </c>
+      <c r="J40" s="2">
         <v>0</v>
       </c>
       <c r="K40">
         <v>1</v>
       </c>
       <c r="L40" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="C41">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D41" t="s">
-        <v>49</v>
-      </c>
-      <c r="E41">
-        <v>395</v>
-      </c>
-      <c r="F41">
-        <v>395</v>
-      </c>
-      <c r="G41">
-        <v>395</v>
-      </c>
-      <c r="H41">
-        <v>395</v>
-      </c>
-      <c r="I41">
-        <v>395</v>
-      </c>
-      <c r="J41">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="E41" s="2">
+        <v>441</v>
+      </c>
+      <c r="F41" s="2">
+        <v>428</v>
+      </c>
+      <c r="G41" s="2">
+        <v>340</v>
+      </c>
+      <c r="H41" s="2">
+        <v>346</v>
+      </c>
+      <c r="I41" s="3">
+        <v>365</v>
+      </c>
+      <c r="J41" s="2">
+        <v>19</v>
       </c>
       <c r="K41">
         <v>1</v>
       </c>
       <c r="L41" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="C42">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D42" t="s">
-        <v>6</v>
-      </c>
-      <c r="E42">
-        <v>441</v>
-      </c>
-      <c r="F42">
-        <v>428</v>
-      </c>
-      <c r="G42">
-        <v>340</v>
-      </c>
-      <c r="H42">
-        <v>346</v>
-      </c>
-      <c r="I42">
-        <v>365</v>
-      </c>
-      <c r="J42">
-        <v>19</v>
+        <v>46</v>
+      </c>
+      <c r="E42" s="2">
+        <v>198</v>
+      </c>
+      <c r="F42" s="2">
+        <v>198</v>
+      </c>
+      <c r="G42" s="2">
+        <v>198</v>
+      </c>
+      <c r="H42" s="2">
+        <v>198</v>
+      </c>
+      <c r="I42" s="3">
+        <v>198</v>
+      </c>
+      <c r="J42" s="2">
+        <v>0</v>
       </c>
       <c r="K42">
         <v>1</v>
@@ -3801,138 +3959,107 @@
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43">
-        <v>67</v>
+        <v>4</v>
       </c>
       <c r="C43">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D43" t="s">
-        <v>46</v>
-      </c>
-      <c r="E43">
-        <v>198</v>
-      </c>
-      <c r="F43">
-        <v>198</v>
-      </c>
-      <c r="G43">
-        <v>198</v>
-      </c>
-      <c r="H43">
-        <v>198</v>
-      </c>
-      <c r="I43">
-        <v>198</v>
-      </c>
-      <c r="J43">
+        <v>2</v>
+      </c>
+      <c r="E43" s="2">
+        <v>150</v>
+      </c>
+      <c r="F43" s="2">
+        <v>150</v>
+      </c>
+      <c r="G43" s="2">
+        <v>150</v>
+      </c>
+      <c r="H43" s="2">
+        <v>150</v>
+      </c>
+      <c r="I43" s="3">
+        <v>150</v>
+      </c>
+      <c r="J43" s="2">
         <v>0</v>
       </c>
       <c r="K43">
         <v>1</v>
       </c>
       <c r="L43" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44">
-        <v>4</v>
+        <v>72</v>
       </c>
       <c r="C44">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D44" t="s">
+        <v>9</v>
+      </c>
+      <c r="E44" s="2">
+        <v>17027</v>
+      </c>
+      <c r="F44" s="2">
+        <v>28037</v>
+      </c>
+      <c r="G44" s="2">
+        <v>27585</v>
+      </c>
+      <c r="H44" s="2">
+        <v>27507</v>
+      </c>
+      <c r="I44" s="3">
+        <v>27541</v>
+      </c>
+      <c r="J44" s="2">
+        <v>34</v>
+      </c>
+      <c r="K44">
         <v>2</v>
-      </c>
-      <c r="E44">
-        <v>150</v>
-      </c>
-      <c r="F44">
-        <v>150</v>
-      </c>
-      <c r="G44">
-        <v>150</v>
-      </c>
-      <c r="H44">
-        <v>150</v>
-      </c>
-      <c r="I44">
-        <v>150</v>
-      </c>
-      <c r="J44">
-        <v>0</v>
-      </c>
-      <c r="K44">
-        <v>1</v>
-      </c>
-      <c r="L44" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="45" spans="2:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B45"/>
       <c r="C45"/>
       <c r="D45" t="s">
-        <v>65</v>
-      </c>
-      <c r="E45">
+        <v>74</v>
+      </c>
+      <c r="E45" s="2">
         <f>SUBTOTAL(109,Table1[2020])</f>
         <v>1543613</v>
       </c>
-      <c r="F45">
+      <c r="F45" s="2">
         <f>SUBTOTAL(109,Table1[2021])</f>
         <v>1558589</v>
       </c>
-      <c r="G45">
+      <c r="G45" s="2">
         <f>SUBTOTAL(109,Table1[2022])</f>
         <v>1563369</v>
       </c>
-      <c r="H45">
+      <c r="H45" s="2">
         <f>SUBTOTAL(109,Table1[2023])</f>
         <v>1564529</v>
       </c>
-      <c r="I45">
+      <c r="I45" s="3">
         <f>SUBTOTAL(109,Table1[2024])</f>
         <v>1566869</v>
       </c>
-      <c r="J45">
+      <c r="J45" s="2">
         <f>SUBTOTAL(109,Table1[change24/23])</f>
         <v>2340</v>
       </c>
-      <c r="K45">
-        <f>SUBTOTAL(109,Table1[Country2])</f>
-        <v>44</v>
-      </c>
+      <c r="K45"/>
       <c r="L45"/>
     </row>
     <row r="46" spans="2:12" x14ac:dyDescent="0.25">
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
-    </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B47" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C47" s="1"/>
-      <c r="D47" s="1">
-        <v>1543613</v>
-      </c>
-      <c r="E47" s="1">
-        <v>1558589</v>
-      </c>
-      <c r="F47" s="1">
-        <v>1563369</v>
-      </c>
-      <c r="G47" s="1">
-        <v>1564529</v>
-      </c>
-      <c r="H47" s="1">
-        <v>1566869</v>
-      </c>
-      <c r="I47" s="1">
-        <v>2340</v>
-      </c>
-      <c r="J47" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>